<commit_message>
Valores obtenidos de practica
</commit_message>
<xml_diff>
--- a/Design/Calc/Convertidor.xlsx
+++ b/Design/Calc/Convertidor.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ignac\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ignac\Desktop\Bidirectional-Buck-DC-DC-converter\Design\Calc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C07217CF-6E04-41DA-B9FD-CBCF21A5D117}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDDF7EC3-DFCC-4E0A-99D4-B7EDEDC677F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{B77F3227-0229-45A8-A261-1E8C49A76F8E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B77F3227-0229-45A8-A261-1E8C49A76F8E}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="94">
   <si>
     <t>ESPECIFICACIONES</t>
   </si>
@@ -243,6 +243,81 @@
   </si>
   <si>
     <t>95.19%</t>
+  </si>
+  <si>
+    <t>Valores de Resistencia</t>
+  </si>
+  <si>
+    <t>Resistencia 10k</t>
+  </si>
+  <si>
+    <t>Resistencia 100k</t>
+  </si>
+  <si>
+    <t>Resistencia 47k</t>
+  </si>
+  <si>
+    <t>Voltaje sensado</t>
+  </si>
+  <si>
+    <t>10k</t>
+  </si>
+  <si>
+    <t>47k</t>
+  </si>
+  <si>
+    <t>14[V]</t>
+  </si>
+  <si>
+    <t>2.45[V]</t>
+  </si>
+  <si>
+    <t>Voltaje de salida</t>
+  </si>
+  <si>
+    <t>Duty Cycle(%)</t>
+  </si>
+  <si>
+    <t>47.14k</t>
+  </si>
+  <si>
+    <t>2.44[V]</t>
+  </si>
+  <si>
+    <t>13.8[V]</t>
+  </si>
+  <si>
+    <t>46.6k</t>
+  </si>
+  <si>
+    <t>9.8k</t>
+  </si>
+  <si>
+    <t>100k</t>
+  </si>
+  <si>
+    <t>110.6k</t>
+  </si>
+  <si>
+    <t>102k</t>
+  </si>
+  <si>
+    <t>27[V]</t>
+  </si>
+  <si>
+    <t>2.3[V]</t>
+  </si>
+  <si>
+    <t>13.9[V]</t>
+  </si>
+  <si>
+    <t>27V]</t>
+  </si>
+  <si>
+    <t>2.48[V]</t>
+  </si>
+  <si>
+    <t>27.1[V]</t>
   </si>
 </sst>
 </file>
@@ -250,7 +325,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="169" formatCode="0.000%"/>
+    <numFmt numFmtId="164" formatCode="0.000%"/>
   </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
@@ -306,7 +381,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -331,8 +406,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -368,20 +449,23 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -396,7 +480,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="169" fontId="0" fillId="3" borderId="1" xfId="1" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="1" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="10" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -404,6 +488,26 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -432,8 +536,8 @@
       <xdr:rowOff>69894</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>512379</xdr:colOff>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>1301921</xdr:colOff>
       <xdr:row>40</xdr:row>
       <xdr:rowOff>60587</xdr:rowOff>
     </xdr:to>
@@ -493,8 +597,8 @@
       <xdr:rowOff>118241</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>183932</xdr:colOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>523619</xdr:colOff>
       <xdr:row>40</xdr:row>
       <xdr:rowOff>157655</xdr:rowOff>
     </xdr:to>
@@ -554,8 +658,8 @@
       <xdr:rowOff>14997</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>378461</xdr:colOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>1168003</xdr:colOff>
       <xdr:row>42</xdr:row>
       <xdr:rowOff>13138</xdr:rowOff>
     </xdr:to>
@@ -652,10 +756,6 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -975,7 +1075,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5558E28-EA4A-4CEC-8A03-B5F73659600E}">
-  <dimension ref="C3:M49"/>
+  <dimension ref="C3:N61"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="5.21875" customWidth="1"/>
@@ -983,28 +1083,31 @@
     <col min="4" max="4" width="22" customWidth="1"/>
     <col min="5" max="5" width="20.88671875" customWidth="1"/>
     <col min="6" max="6" width="25.6640625" customWidth="1"/>
-    <col min="9" max="9" width="6.5546875" customWidth="1"/>
+    <col min="7" max="7" width="23.33203125" customWidth="1"/>
+    <col min="8" max="8" width="24.88671875" customWidth="1"/>
+    <col min="9" max="9" width="25.6640625" customWidth="1"/>
     <col min="10" max="10" width="26.77734375" customWidth="1"/>
     <col min="11" max="11" width="24.109375" customWidth="1"/>
     <col min="12" max="12" width="22.44140625" customWidth="1"/>
     <col min="13" max="13" width="22.5546875" customWidth="1"/>
+    <col min="14" max="15" width="21.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="3:13" ht="18" x14ac:dyDescent="0.35">
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
+      <c r="D3" s="15"/>
+      <c r="E3" s="15"/>
     </row>
     <row r="5" spans="3:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="3" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1064,40 +1167,40 @@
       </c>
     </row>
     <row r="14" spans="3:13" ht="18" x14ac:dyDescent="0.35">
-      <c r="C14" s="3" t="s">
+      <c r="C14" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="J14" s="3" t="s">
+      <c r="D14" s="15"/>
+      <c r="E14" s="15"/>
+      <c r="J14" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="K14" s="2"/>
-      <c r="L14" s="2"/>
+      <c r="K14" s="15"/>
+      <c r="L14" s="15"/>
     </row>
     <row r="16" spans="3:13" ht="18" x14ac:dyDescent="0.35">
-      <c r="C16" s="7" t="s">
+      <c r="C16" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="D16" s="7" t="s">
+      <c r="D16" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="E16" s="7" t="s">
+      <c r="E16" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="F16" s="7" t="s">
+      <c r="F16" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J16" s="7" t="s">
+      <c r="J16" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="K16" s="7" t="s">
+      <c r="K16" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="L16" s="7" t="s">
+      <c r="L16" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="M16" s="7" t="s">
+      <c r="M16" s="5" t="s">
         <v>20</v>
       </c>
     </row>
@@ -1105,25 +1208,25 @@
       <c r="C17" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D17" s="9">
+      <c r="D17" s="7">
         <v>0.01</v>
       </c>
-      <c r="E17" s="9" t="s">
+      <c r="E17" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="F17" s="12">
+      <c r="F17" s="10">
         <v>1.0030000000000001E-2</v>
       </c>
       <c r="J17" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="K17" s="9">
+      <c r="K17" s="7">
         <v>0.01</v>
       </c>
-      <c r="L17" s="9" t="s">
+      <c r="L17" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="M17" s="12" t="s">
+      <c r="M17" s="10" t="s">
         <v>57</v>
       </c>
     </row>
@@ -1131,25 +1234,25 @@
       <c r="C18" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="D18" s="9">
+      <c r="D18" s="7">
         <v>0.3</v>
       </c>
-      <c r="E18" s="9">
+      <c r="E18" s="7">
         <v>0.28999999999999998</v>
       </c>
-      <c r="F18" s="13">
+      <c r="F18" s="11">
         <v>0.17319999999999999</v>
       </c>
       <c r="J18" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="K18" s="9">
+      <c r="K18" s="7">
         <v>0.3</v>
       </c>
-      <c r="L18" s="9" t="s">
+      <c r="L18" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="M18" s="13" t="s">
+      <c r="M18" s="11" t="s">
         <v>56</v>
       </c>
     </row>
@@ -1157,25 +1260,25 @@
       <c r="C19" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="D19" s="10" t="s">
+      <c r="D19" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="E19" s="10" t="s">
+      <c r="E19" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="F19" s="10" t="s">
+      <c r="F19" s="8" t="s">
         <v>28</v>
       </c>
       <c r="J19" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="K19" s="10" t="s">
+      <c r="K19" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="L19" s="10" t="s">
+      <c r="L19" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="M19" s="10" t="s">
+      <c r="M19" s="8" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1183,25 +1286,25 @@
       <c r="C20" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D20" s="10" t="s">
+      <c r="D20" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E20" s="10" t="s">
+      <c r="E20" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="F20" s="10" t="s">
+      <c r="F20" s="8" t="s">
         <v>38</v>
       </c>
       <c r="J20" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="K20" s="10" t="s">
+      <c r="K20" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="L20" s="10" t="s">
+      <c r="L20" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="M20" s="10" t="s">
+      <c r="M20" s="8" t="s">
         <v>50</v>
       </c>
     </row>
@@ -1209,25 +1312,25 @@
       <c r="C21" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="D21" s="10" t="s">
+      <c r="D21" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="E21" s="10" t="s">
+      <c r="E21" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="F21" s="10" t="s">
+      <c r="F21" s="8" t="s">
         <v>40</v>
       </c>
       <c r="J21" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="K21" s="10" t="s">
+      <c r="K21" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="L21" s="10" t="s">
+      <c r="L21" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="M21" s="10" t="s">
+      <c r="M21" s="8" t="s">
         <v>51</v>
       </c>
     </row>
@@ -1235,51 +1338,51 @@
       <c r="C22" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="D22" s="10" t="s">
+      <c r="D22" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="E22" s="10" t="s">
+      <c r="E22" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="F22" s="10" t="s">
+      <c r="F22" s="8" t="s">
         <v>37</v>
       </c>
       <c r="J22" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="K22" s="10" t="s">
+      <c r="K22" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="L22" s="10" t="s">
+      <c r="L22" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="M22" s="10" t="s">
+      <c r="M22" s="8" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="23" spans="3:13" x14ac:dyDescent="0.3">
-      <c r="C23" s="8" t="s">
+      <c r="C23" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="D23" s="10" t="s">
+      <c r="D23" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="E23" s="9">
+      <c r="E23" s="7">
         <v>0.61</v>
       </c>
-      <c r="F23" s="9">
+      <c r="F23" s="7">
         <v>0.65</v>
       </c>
-      <c r="J23" s="8" t="s">
+      <c r="J23" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="K23" s="10" t="s">
+      <c r="K23" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="L23" s="9">
+      <c r="L23" s="7">
         <v>0.6</v>
       </c>
-      <c r="M23" s="9" t="s">
+      <c r="M23" s="7" t="s">
         <v>52</v>
       </c>
     </row>
@@ -1287,70 +1390,70 @@
       <c r="C24" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="D24" s="9" t="s">
+      <c r="D24" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="E24" s="10" t="s">
+      <c r="E24" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="F24" s="10" t="s">
+      <c r="F24" s="8" t="s">
         <v>55</v>
       </c>
       <c r="J24" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="K24" s="9" t="s">
+      <c r="K24" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="L24" s="10" t="s">
+      <c r="L24" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="M24" s="10" t="s">
+      <c r="M24" s="8" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="25" spans="3:13" x14ac:dyDescent="0.3">
-      <c r="C25" s="11" t="s">
+      <c r="C25" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D25" s="9">
+      <c r="D25" s="7">
         <v>1</v>
       </c>
-      <c r="E25" s="10" t="s">
+      <c r="E25" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="F25" s="9" t="s">
+      <c r="F25" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="J25" s="11" t="s">
+      <c r="J25" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="K25" s="9">
+      <c r="K25" s="7">
         <v>1</v>
       </c>
-      <c r="L25" s="10" t="s">
+      <c r="L25" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="M25" s="9" t="s">
+      <c r="M25" s="7" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="28" spans="3:13" ht="21" x14ac:dyDescent="0.4">
-      <c r="C28" s="15" t="s">
+      <c r="C28" s="13" t="s">
         <v>59</v>
       </c>
-      <c r="F28" s="14" t="s">
+      <c r="F28" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="J28" s="14" t="s">
+      <c r="J28" s="12" t="s">
         <v>59</v>
       </c>
-      <c r="M28" s="14" t="s">
+      <c r="M28" s="12" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="45" spans="3:4" x14ac:dyDescent="0.3">
-      <c r="C45" s="6" t="s">
+      <c r="C45" s="4" t="s">
         <v>62</v>
       </c>
     </row>
@@ -1378,15 +1481,236 @@
         <v>66</v>
       </c>
     </row>
-    <row r="49" spans="3:4" x14ac:dyDescent="0.3">
+    <row r="49" spans="3:14" x14ac:dyDescent="0.3">
       <c r="C49" s="1"/>
       <c r="D49" s="1"/>
     </row>
+    <row r="50" spans="3:14" ht="18" x14ac:dyDescent="0.35">
+      <c r="F50" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="G50" s="15"/>
+      <c r="H50" s="15"/>
+      <c r="K50" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="L50" s="15"/>
+      <c r="M50" s="15"/>
+    </row>
+    <row r="52" spans="3:14" x14ac:dyDescent="0.3">
+      <c r="C52" s="16" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="53" spans="3:14" ht="18" x14ac:dyDescent="0.35">
+      <c r="C53" s="1"/>
+      <c r="D53" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="F53" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G53" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="H53" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="I53" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="K53" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="L53" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="M53" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="N53" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="54" spans="3:14" x14ac:dyDescent="0.3">
+      <c r="C54" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D54" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="F54" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="G54" s="17" t="s">
+        <v>74</v>
+      </c>
+      <c r="H54" s="17" t="s">
+        <v>74</v>
+      </c>
+      <c r="I54" s="17" t="s">
+        <v>84</v>
+      </c>
+      <c r="K54" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="L54" s="17" t="s">
+        <v>74</v>
+      </c>
+      <c r="M54" s="17" t="s">
+        <v>74</v>
+      </c>
+      <c r="N54" s="17" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="55" spans="3:14" x14ac:dyDescent="0.3">
+      <c r="C55" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D55" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="F55" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="G55" s="17" t="s">
+        <v>80</v>
+      </c>
+      <c r="H55" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="I55" s="17" t="s">
+        <v>83</v>
+      </c>
+      <c r="K55" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="L55" s="17" t="s">
+        <v>87</v>
+      </c>
+      <c r="M55" s="17" t="s">
+        <v>85</v>
+      </c>
+      <c r="N55" s="17" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="56" spans="3:14" x14ac:dyDescent="0.3">
+      <c r="C56" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D56" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="F56" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="G56" s="17" t="s">
+        <v>77</v>
+      </c>
+      <c r="H56" s="17" t="s">
+        <v>81</v>
+      </c>
+      <c r="I56" s="17" t="s">
+        <v>89</v>
+      </c>
+      <c r="K56" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="L56" s="17" t="s">
+        <v>77</v>
+      </c>
+      <c r="M56" s="17" t="s">
+        <v>77</v>
+      </c>
+      <c r="N56" s="17" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="57" spans="3:14" x14ac:dyDescent="0.3">
+      <c r="C57" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D57" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="F57" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="G57" s="18" t="s">
+        <v>76</v>
+      </c>
+      <c r="H57" s="17" t="s">
+        <v>82</v>
+      </c>
+      <c r="I57" s="17" t="s">
+        <v>90</v>
+      </c>
+      <c r="K57" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="L57" s="18" t="s">
+        <v>88</v>
+      </c>
+      <c r="M57" s="17" t="s">
+        <v>91</v>
+      </c>
+      <c r="N57" s="17" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="58" spans="3:14" x14ac:dyDescent="0.3">
+      <c r="F58" s="19" t="s">
+        <v>79</v>
+      </c>
+      <c r="G58" s="20">
+        <v>0.6</v>
+      </c>
+      <c r="H58" s="20">
+        <v>0.61</v>
+      </c>
+      <c r="I58" s="20">
+        <v>0.69</v>
+      </c>
+      <c r="K58" s="19" t="s">
+        <v>79</v>
+      </c>
+      <c r="L58" s="23" t="s">
+        <v>43</v>
+      </c>
+      <c r="M58" s="20">
+        <v>0.59</v>
+      </c>
+      <c r="N58" s="20">
+        <v>0.67</v>
+      </c>
+    </row>
+    <row r="59" spans="3:14" x14ac:dyDescent="0.3">
+      <c r="F59" s="22"/>
+      <c r="G59" s="22"/>
+      <c r="H59" s="22"/>
+      <c r="I59" s="22"/>
+    </row>
+    <row r="60" spans="3:14" x14ac:dyDescent="0.3">
+      <c r="F60" s="21"/>
+      <c r="G60" s="21"/>
+      <c r="H60" s="21"/>
+      <c r="I60" s="21"/>
+    </row>
+    <row r="61" spans="3:14" x14ac:dyDescent="0.3">
+      <c r="F61" s="21"/>
+      <c r="G61" s="21"/>
+      <c r="H61" s="21"/>
+      <c r="I61" s="21"/>
+    </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="5">
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="C14:E14"/>
     <mergeCell ref="J14:L14"/>
+    <mergeCell ref="F50:H50"/>
+    <mergeCell ref="K50:M50"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -1642,20 +1966,20 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="a96d87df-68fc-4a03-8684-6db9968eb191" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="a96d87df-68fc-4a03-8684-6db9968eb191" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1678,14 +2002,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FA3761E3-028C-44E9-B520-877AF5DBE492}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C8B83733-5969-4545-9D8F-F85C281218A0}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
@@ -1700,4 +2016,12 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FA3761E3-028C-44E9-B520-877AF5DBE492}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>